<commit_message>
chore(auto): review daily 2026-05-25
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models.xlsx
+++ b/Model_Navigate/data/Object-Models.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q406"/>
+  <dimension ref="A1:Q405"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23014,61 +23014,6 @@
         </is>
       </c>
     </row>
-    <row r="406">
-      <c r="A406" t="inlineStr">
-        <is>
-          <t>昇腾AgentInfra</t>
-        </is>
-      </c>
-      <c r="B406" t="inlineStr"/>
-      <c r="C406" t="inlineStr"/>
-      <c r="D406" t="inlineStr">
-        <is>
-          <t>华为</t>
-        </is>
-      </c>
-      <c r="E406" t="inlineStr">
-        <is>
-          <t>国内</t>
-        </is>
-      </c>
-      <c r="F406" t="inlineStr"/>
-      <c r="G406" t="inlineStr"/>
-      <c r="H406" t="inlineStr">
-        <is>
-          <t>agent runtime infrastructure</t>
-        </is>
-      </c>
-      <c r="I406" t="inlineStr"/>
-      <c r="J406" t="inlineStr"/>
-      <c r="K406" t="inlineStr"/>
-      <c r="L406" t="inlineStr">
-        <is>
-          <t>华为鲲鹏昇腾开发者大会上发布的智能体原生运行环境，作为‘鲲鹏硬核算力 + openEuler异构系统 + AgentInfra’三层架构核心组件全面开源。</t>
-        </is>
-      </c>
-      <c r="M406" t="inlineStr">
-        <is>
-          <t>2026-05-24</t>
-        </is>
-      </c>
-      <c r="N406" t="inlineStr">
-        <is>
-          <t>2026-05-25 02:13</t>
-        </is>
-      </c>
-      <c r="O406" t="inlineStr"/>
-      <c r="P406" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="Q406" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-05-26
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models.xlsx
+++ b/Model_Navigate/data/Object-Models.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q405"/>
+  <dimension ref="A1:Q406"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23014,6 +23014,65 @@
         </is>
       </c>
     </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>昇腾AgentInfra</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr"/>
+      <c r="C406" t="inlineStr"/>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>华为</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F406" t="inlineStr"/>
+      <c r="G406" t="inlineStr"/>
+      <c r="H406" t="inlineStr">
+        <is>
+          <t>agent runtime infrastructure</t>
+        </is>
+      </c>
+      <c r="I406" t="inlineStr"/>
+      <c r="J406" t="inlineStr"/>
+      <c r="K406" t="inlineStr"/>
+      <c r="L406" t="inlineStr">
+        <is>
+          <t>华为鲲鹏昇腾开发者大会上发布的智能体原生运行环境，作为‘鲲鹏硬核算力 + openEuler异构系统 + AgentInfra’三层架构核心组件全面开源。</t>
+        </is>
+      </c>
+      <c r="M406" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="N406" t="inlineStr">
+        <is>
+          <t>2026-05-25 02:13</t>
+        </is>
+      </c>
+      <c r="O406" t="inlineStr">
+        <is>
+          <t>2026-05-26 02:03</t>
+        </is>
+      </c>
+      <c r="P406" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Q406" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5建议删除(中置信)待人工确认 — 建议删除：产品泛称无版本号; 非具体模型条目：昇腾AgentInfra更像智能体运行环境/基础设施组件，不属于模型名称; 模型名称缺少明确版本号或型号; 类型分类不应归为模型，应归为智能体基础设施/运行时</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(auto): review daily 2026-05-27
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models.xlsx
+++ b/Model_Navigate/data/Object-Models.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q413"/>
+  <dimension ref="A1:Q412"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23360,14 +23360,14 @@
     <row r="411">
       <c r="A411" t="inlineStr">
         <is>
-          <t>Grok V9-Medium</t>
+          <t>MiniCPM5-1B</t>
         </is>
       </c>
       <c r="B411" t="inlineStr"/>
       <c r="C411" t="inlineStr"/>
       <c r="D411" t="inlineStr">
         <is>
-          <t>SpaceXAI (xAI)</t>
+          <t>OpenBMB</t>
         </is>
       </c>
       <c r="E411" t="inlineStr">
@@ -23379,7 +23379,7 @@
       <c r="G411" t="inlineStr"/>
       <c r="H411" t="inlineStr">
         <is>
-          <t>大语言模型</t>
+          <t>小规模混合推理大语言模型</t>
         </is>
       </c>
       <c r="I411" t="inlineStr"/>
@@ -23387,7 +23387,7 @@
       <c r="K411" t="inlineStr"/>
       <c r="L411" t="inlineStr">
         <is>
-          <t>1.5T参数基础模型，已完成训练并进入微调阶段，专为复杂编程任务优化，预计2–3周内公开发布，年底将开源0.5T版本。</t>
+          <t>10.8亿参数开源模型，登顶Artificial Analysis小模型榜单（17.9分），支持INT4量化（约0.5GB），可在手机、浏览器及CPU本地运行。</t>
         </is>
       </c>
       <c r="M411" t="inlineStr">
@@ -23415,14 +23415,14 @@
     <row r="412">
       <c r="A412" t="inlineStr">
         <is>
-          <t>MiniCPM5-1B</t>
+          <t>Gemini 3.5 Flash (Low)</t>
         </is>
       </c>
       <c r="B412" t="inlineStr"/>
       <c r="C412" t="inlineStr"/>
       <c r="D412" t="inlineStr">
         <is>
-          <t>OpenBMB</t>
+          <t>Google / DeepMind</t>
         </is>
       </c>
       <c r="E412" t="inlineStr">
@@ -23434,7 +23434,7 @@
       <c r="G412" t="inlineStr"/>
       <c r="H412" t="inlineStr">
         <is>
-          <t>小规模混合推理大语言模型</t>
+          <t>轻量级多模态大语言模型</t>
         </is>
       </c>
       <c r="I412" t="inlineStr"/>
@@ -23442,7 +23442,7 @@
       <c r="K412" t="inlineStr"/>
       <c r="L412" t="inlineStr">
         <is>
-          <t>10.8亿参数开源模型，登顶Artificial Analysis小模型榜单（17.9分），支持INT4量化（约0.5GB），可在手机、浏览器及CPU本地运行。</t>
+          <t>Antigravity平台新增的低延迟、低成本推理变体，面向高并发轻负载场景优化，为Gemini 3.5系列首次推出的‘Flash’分级型号。</t>
         </is>
       </c>
       <c r="M412" t="inlineStr">
@@ -23462,61 +23462,6 @@
         </is>
       </c>
       <c r="Q412" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-    </row>
-    <row r="413">
-      <c r="A413" t="inlineStr">
-        <is>
-          <t>Gemini 3.5 Flash (Low)</t>
-        </is>
-      </c>
-      <c r="B413" t="inlineStr"/>
-      <c r="C413" t="inlineStr"/>
-      <c r="D413" t="inlineStr">
-        <is>
-          <t>Google / DeepMind</t>
-        </is>
-      </c>
-      <c r="E413" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F413" t="inlineStr"/>
-      <c r="G413" t="inlineStr"/>
-      <c r="H413" t="inlineStr">
-        <is>
-          <t>轻量级多模态大语言模型</t>
-        </is>
-      </c>
-      <c r="I413" t="inlineStr"/>
-      <c r="J413" t="inlineStr"/>
-      <c r="K413" t="inlineStr"/>
-      <c r="L413" t="inlineStr">
-        <is>
-          <t>Antigravity平台新增的低延迟、低成本推理变体，面向高并发轻负载场景优化，为Gemini 3.5系列首次推出的‘Flash’分级型号。</t>
-        </is>
-      </c>
-      <c r="M413" t="inlineStr">
-        <is>
-          <t>2026-05-26</t>
-        </is>
-      </c>
-      <c r="N413" t="inlineStr">
-        <is>
-          <t>2026-05-27 02:12</t>
-        </is>
-      </c>
-      <c r="O413" t="inlineStr"/>
-      <c r="P413" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="Q413" t="inlineStr">
         <is>
           <t>待核实（LLM交叉巡检发现）</t>
         </is>

</xml_diff>

<commit_message>
chore(auto): review daily 2026-05-29
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models.xlsx
+++ b/Model_Navigate/data/Object-Models.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q428"/>
+  <dimension ref="A1:Q427"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24172,26 +24172,26 @@
     <row r="425">
       <c r="A425" t="inlineStr">
         <is>
-          <t>Meta One Plus / Meta One Premium</t>
+          <t>MuleRun</t>
         </is>
       </c>
       <c r="B425" t="inlineStr"/>
       <c r="C425" t="inlineStr"/>
       <c r="D425" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>阿里巴巴/通义</t>
         </is>
       </c>
       <c r="E425" t="inlineStr">
         <is>
-          <t>国外</t>
+          <t>国内</t>
         </is>
       </c>
       <c r="F425" t="inlineStr"/>
       <c r="G425" t="inlineStr"/>
       <c r="H425" t="inlineStr">
         <is>
-          <t>AI智能体（聊天机器人服务）</t>
+          <t>AI智能体框架</t>
         </is>
       </c>
       <c r="I425" t="inlineStr"/>
@@ -24199,12 +24199,12 @@
       <c r="K425" t="inlineStr"/>
       <c r="L425" t="inlineStr">
         <is>
-          <t>Meta于2026年5月28日宣布下月起测试的付费AI智能体订阅服务，覆盖Facebook、Instagram、WhatsApp和Meta AI，提供分级AI生成与推理能力，标志其从免费AI助手转向商业化智能体生态。</t>
+          <t>阿里云于2026年5月26日在新加坡Qwen Cloud发布会上推出的轻量级、可编排AI智能体运行时框架，专为低延迟Agent工作流设计，支持千问云Skills原生调度。</t>
         </is>
       </c>
       <c r="M425" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="N425" t="inlineStr">
@@ -24227,7 +24227,7 @@
     <row r="426">
       <c r="A426" t="inlineStr">
         <is>
-          <t>MuleRun</t>
+          <t>Qoder</t>
         </is>
       </c>
       <c r="B426" t="inlineStr"/>
@@ -24246,7 +24246,7 @@
       <c r="G426" t="inlineStr"/>
       <c r="H426" t="inlineStr">
         <is>
-          <t>AI智能体框架</t>
+          <t>智能体编程平台</t>
         </is>
       </c>
       <c r="I426" t="inlineStr"/>
@@ -24254,7 +24254,7 @@
       <c r="K426" t="inlineStr"/>
       <c r="L426" t="inlineStr">
         <is>
-          <t>阿里云于2026年5月26日在新加坡Qwen Cloud发布会上推出的轻量级、可编排AI智能体运行时框架，专为低延迟Agent工作流设计，支持千问云Skills原生调度。</t>
+          <t>阿里云同步发布的面向开发者的新一代智能体编程平台，支持自然语言定义Agent行为、可视化调试与一键部署至千问云，是Qwen3.7-Max的核心配套开发环境。</t>
         </is>
       </c>
       <c r="M426" t="inlineStr">
@@ -24282,26 +24282,26 @@
     <row r="427">
       <c r="A427" t="inlineStr">
         <is>
-          <t>Qoder</t>
+          <t>稀宇极智MoE大模型（未公开命名）</t>
         </is>
       </c>
       <c r="B427" t="inlineStr"/>
       <c r="C427" t="inlineStr"/>
       <c r="D427" t="inlineStr">
         <is>
-          <t>阿里巴巴/通义</t>
+          <t>上海稀宇极智科技有限公司</t>
         </is>
       </c>
       <c r="E427" t="inlineStr">
         <is>
-          <t>国内</t>
+          <t>国外</t>
         </is>
       </c>
       <c r="F427" t="inlineStr"/>
       <c r="G427" t="inlineStr"/>
       <c r="H427" t="inlineStr">
         <is>
-          <t>智能体编程平台</t>
+          <t>混合专家系统（MoE）大语言模型</t>
         </is>
       </c>
       <c r="I427" t="inlineStr"/>
@@ -24309,12 +24309,12 @@
       <c r="K427" t="inlineStr"/>
       <c r="L427" t="inlineStr">
         <is>
-          <t>阿里云同步发布的面向开发者的新一代智能体编程平台，支持自然语言定义Agent行为、可视化调试与一键部署至千问云，是Qwen3.7-Max的核心配套开发环境。</t>
+          <t>稀宇极智于2026年5月28日国务院新闻办中外记者见面会上确认发布的国内首个全自研MoE架构大模型，以不到行业巨头1%算力成本实现顶尖性能，覆盖文本理解、语音合成、视频生成及智能体全栈能力。</t>
         </is>
       </c>
       <c r="M427" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="N427" t="inlineStr">
@@ -24329,61 +24329,6 @@
         </is>
       </c>
       <c r="Q427" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-    </row>
-    <row r="428">
-      <c r="A428" t="inlineStr">
-        <is>
-          <t>稀宇极智MoE大模型（未公开命名）</t>
-        </is>
-      </c>
-      <c r="B428" t="inlineStr"/>
-      <c r="C428" t="inlineStr"/>
-      <c r="D428" t="inlineStr">
-        <is>
-          <t>上海稀宇极智科技有限公司</t>
-        </is>
-      </c>
-      <c r="E428" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F428" t="inlineStr"/>
-      <c r="G428" t="inlineStr"/>
-      <c r="H428" t="inlineStr">
-        <is>
-          <t>混合专家系统（MoE）大语言模型</t>
-        </is>
-      </c>
-      <c r="I428" t="inlineStr"/>
-      <c r="J428" t="inlineStr"/>
-      <c r="K428" t="inlineStr"/>
-      <c r="L428" t="inlineStr">
-        <is>
-          <t>稀宇极智于2026年5月28日国务院新闻办中外记者见面会上确认发布的国内首个全自研MoE架构大模型，以不到行业巨头1%算力成本实现顶尖性能，覆盖文本理解、语音合成、视频生成及智能体全栈能力。</t>
-        </is>
-      </c>
-      <c r="M428" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="N428" t="inlineStr">
-        <is>
-          <t>2026-05-29 02:04</t>
-        </is>
-      </c>
-      <c r="O428" t="inlineStr"/>
-      <c r="P428" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="Q428" t="inlineStr">
         <is>
           <t>待核实（LLM交叉巡检发现）</t>
         </is>

</xml_diff>

<commit_message>
chore(auto): review daily 2026-06-03
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models.xlsx
+++ b/Model_Navigate/data/Object-Models.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q435"/>
+  <dimension ref="A1:Q434"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24755,61 +24755,6 @@
         </is>
       </c>
     </row>
-    <row r="435">
-      <c r="A435" t="inlineStr">
-        <is>
-          <t>LobsterAI Image-Video Matrix</t>
-        </is>
-      </c>
-      <c r="B435" t="inlineStr"/>
-      <c r="C435" t="inlineStr"/>
-      <c r="D435" t="inlineStr">
-        <is>
-          <t>LobsterAI</t>
-        </is>
-      </c>
-      <c r="E435" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F435" t="inlineStr"/>
-      <c r="G435" t="inlineStr"/>
-      <c r="H435" t="inlineStr">
-        <is>
-          <t>图像/视频生成大模型矩阵</t>
-        </is>
-      </c>
-      <c r="I435" t="inlineStr"/>
-      <c r="J435" t="inlineStr"/>
-      <c r="K435" t="inlineStr"/>
-      <c r="L435" t="inlineStr">
-        <is>
-          <t>LobsterAI发布的多分辨率、多时长视频与高保真图像协同生成模型集合。</t>
-        </is>
-      </c>
-      <c r="M435" t="inlineStr">
-        <is>
-          <t>2026-06-02</t>
-        </is>
-      </c>
-      <c r="N435" t="inlineStr">
-        <is>
-          <t>2026-06-03 02:40</t>
-        </is>
-      </c>
-      <c r="O435" t="inlineStr"/>
-      <c r="P435" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="Q435" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(auto): review daily 2026-06-04
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models.xlsx
+++ b/Model_Navigate/data/Object-Models.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q442"/>
+  <dimension ref="A1:Q440"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25037,14 +25037,14 @@
     <row r="440">
       <c r="A440" t="inlineStr">
         <is>
-          <t>MAI-Multimodal-Agent-1</t>
+          <t>Mayo-Medical-LLM (codename: MedSage)</t>
         </is>
       </c>
       <c r="B440" t="inlineStr"/>
       <c r="C440" t="inlineStr"/>
       <c r="D440" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Mayo Clinic &amp; Microsoft</t>
         </is>
       </c>
       <c r="E440" t="inlineStr">
@@ -25056,7 +25056,7 @@
       <c r="G440" t="inlineStr"/>
       <c r="H440" t="inlineStr">
         <is>
-          <t>自主智能体（Agent）系统</t>
+          <t>医疗垂直领域大语言模型</t>
         </is>
       </c>
       <c r="I440" t="inlineStr"/>
@@ -25064,7 +25064,7 @@
       <c r="K440" t="inlineStr"/>
       <c r="L440" t="inlineStr">
         <is>
-          <t>基于 MAI 系列模型构建的首个端到端可执行智能体框架，支持任务规划、工具调用、Web IQ 搜索协同与长期记忆，面向企业自动化场景开放 SDK。</t>
+          <t>梅奥诊所与微软联合发布、由梅奥持有主权的临床级 AI 模型，基于去标识化真实世界健康数据训练，专注临床推理与诊疗辅助，尚未开源或商用。</t>
         </is>
       </c>
       <c r="M440" t="inlineStr">
@@ -25084,116 +25084,6 @@
         </is>
       </c>
       <c r="Q440" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-    </row>
-    <row r="441">
-      <c r="A441" t="inlineStr">
-        <is>
-          <t>Web IQ</t>
-        </is>
-      </c>
-      <c r="B441" t="inlineStr"/>
-      <c r="C441" t="inlineStr"/>
-      <c r="D441" t="inlineStr">
-        <is>
-          <t>Microsoft</t>
-        </is>
-      </c>
-      <c r="E441" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F441" t="inlineStr"/>
-      <c r="G441" t="inlineStr"/>
-      <c r="H441" t="inlineStr">
-        <is>
-          <t>AI智能体专用搜索 API 服务</t>
-        </is>
-      </c>
-      <c r="I441" t="inlineStr"/>
-      <c r="J441" t="inlineStr"/>
-      <c r="K441" t="inlineStr"/>
-      <c r="L441" t="inlineStr">
-        <is>
-          <t>微软推出的面向 AI 智能体的语义化网络检索服务，提供带 grounding 的结构化网页、新闻、图片、视频内容，非面向人类的传统搜索引擎。</t>
-        </is>
-      </c>
-      <c r="M441" t="inlineStr">
-        <is>
-          <t>2026-06-03</t>
-        </is>
-      </c>
-      <c r="N441" t="inlineStr">
-        <is>
-          <t>2026-06-04 02:36</t>
-        </is>
-      </c>
-      <c r="O441" t="inlineStr"/>
-      <c r="P441" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="Q441" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-    </row>
-    <row r="442">
-      <c r="A442" t="inlineStr">
-        <is>
-          <t>Mayo-Medical-LLM (codename: MedSage)</t>
-        </is>
-      </c>
-      <c r="B442" t="inlineStr"/>
-      <c r="C442" t="inlineStr"/>
-      <c r="D442" t="inlineStr">
-        <is>
-          <t>Mayo Clinic &amp; Microsoft</t>
-        </is>
-      </c>
-      <c r="E442" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F442" t="inlineStr"/>
-      <c r="G442" t="inlineStr"/>
-      <c r="H442" t="inlineStr">
-        <is>
-          <t>医疗垂直领域大语言模型</t>
-        </is>
-      </c>
-      <c r="I442" t="inlineStr"/>
-      <c r="J442" t="inlineStr"/>
-      <c r="K442" t="inlineStr"/>
-      <c r="L442" t="inlineStr">
-        <is>
-          <t>梅奥诊所与微软联合发布、由梅奥持有主权的临床级 AI 模型，基于去标识化真实世界健康数据训练，专注临床推理与诊疗辅助，尚未开源或商用。</t>
-        </is>
-      </c>
-      <c r="M442" t="inlineStr">
-        <is>
-          <t>2026-06-03</t>
-        </is>
-      </c>
-      <c r="N442" t="inlineStr">
-        <is>
-          <t>2026-06-04 02:36</t>
-        </is>
-      </c>
-      <c r="O442" t="inlineStr"/>
-      <c r="P442" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="Q442" t="inlineStr">
         <is>
           <t>待核实（LLM交叉巡检发现）</t>
         </is>

</xml_diff>

<commit_message>
chore(auto): review daily 2026-06-08
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models.xlsx
+++ b/Model_Navigate/data/Object-Models.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q485"/>
+  <dimension ref="A1:Q483"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27516,26 +27516,26 @@
     <row r="481">
       <c r="A481" t="inlineStr">
         <is>
-          <t>Claude 4.0</t>
+          <t>Qwen-Agent v3.2</t>
         </is>
       </c>
       <c r="B481" t="inlineStr"/>
       <c r="C481" t="inlineStr"/>
       <c r="D481" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>阿里巴巴/通义实验室</t>
         </is>
       </c>
       <c r="E481" t="inlineStr">
         <is>
-          <t>国外</t>
+          <t>国内</t>
         </is>
       </c>
       <c r="F481" t="inlineStr"/>
       <c r="G481" t="inlineStr"/>
       <c r="H481" t="inlineStr">
         <is>
-          <t>大语言模型</t>
+          <t>AI智能体系统</t>
         </is>
       </c>
       <c r="I481" t="inlineStr"/>
@@ -27543,12 +27543,12 @@
       <c r="K481" t="inlineStr"/>
       <c r="L481" t="inlineStr">
         <is>
-          <t>Anthropic正式发布Claude 4.0，宣称在1M上下文处理、工具调用稳定性及多智能体协同协议（MCP）原生支持方面实现突破，面向企业级Agent工作流深度优化</t>
+          <t>基于CUA范式构建的生产级Agent框架，支持自动Tool编排、跨会话状态持久化与可验证决策链，已接入钉钉与阿里云百炼平台</t>
         </is>
       </c>
       <c r="M481" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="N481" t="inlineStr">
@@ -27571,14 +27571,14 @@
     <row r="482">
       <c r="A482" t="inlineStr">
         <is>
-          <t>CUA (Contextual Utility Alignment) Training Framework</t>
+          <t>Kimi K2 Thinking</t>
         </is>
       </c>
       <c r="B482" t="inlineStr"/>
       <c r="C482" t="inlineStr"/>
       <c r="D482" t="inlineStr">
         <is>
-          <t>复旦大学 × 通义实验室</t>
+          <t>月之暗面 (Moonshot AI)</t>
         </is>
       </c>
       <c r="E482" t="inlineStr">
@@ -27590,7 +27590,7 @@
       <c r="G482" t="inlineStr"/>
       <c r="H482" t="inlineStr">
         <is>
-          <t>智能体训练范式 / 方法论</t>
+          <t>推理增强型思考模型</t>
         </is>
       </c>
       <c r="I482" t="inlineStr"/>
@@ -27598,12 +27598,12 @@
       <c r="K482" t="inlineStr"/>
       <c r="L482" t="inlineStr">
         <is>
-          <t>提出全新CUA训练范式，解决Agent在复杂Tool选择中的效用对齐问题，非单一模型但已集成至通义千问Qwen-Agent v3.2（同期上线）</t>
+          <t>虽发布于2025年11月，但在2026年5月30日被量子位等媒体重点报道其‘300轮自主工具调用’能力，并作为K2系列核心组件在2026年5月下旬技术峰会中全面演示，属搜索窗口内关键再曝光模型</t>
         </is>
       </c>
       <c r="M482" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2025-11-01</t>
         </is>
       </c>
       <c r="N482" t="inlineStr">
@@ -27626,26 +27626,26 @@
     <row r="483">
       <c r="A483" t="inlineStr">
         <is>
-          <t>Qwen-Agent v3.2</t>
+          <t>Gemini 3.0</t>
         </is>
       </c>
       <c r="B483" t="inlineStr"/>
       <c r="C483" t="inlineStr"/>
       <c r="D483" t="inlineStr">
         <is>
-          <t>阿里巴巴/通义实验室</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="E483" t="inlineStr">
         <is>
-          <t>国内</t>
+          <t>国外</t>
         </is>
       </c>
       <c r="F483" t="inlineStr"/>
       <c r="G483" t="inlineStr"/>
       <c r="H483" t="inlineStr">
         <is>
-          <t>AI智能体系统</t>
+          <t>多模态大模型</t>
         </is>
       </c>
       <c r="I483" t="inlineStr"/>
@@ -27653,12 +27653,12 @@
       <c r="K483" t="inlineStr"/>
       <c r="L483" t="inlineStr">
         <is>
-          <t>基于CUA范式构建的生产级Agent框架，支持自动Tool编排、跨会话状态持久化与可验证决策链，已接入钉钉与阿里云百炼平台</t>
+          <t>Google正式发布Gemini 3.0，原生支持视频帧级推理、实时语音-文本联合规划，并深度集成Antigravity IDE，为2026年5月底前最新多模态基座模型（权威信源确认其GA发布于5月20日，5月29–31日密集应用披露）</t>
         </is>
       </c>
       <c r="M483" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="N483" t="inlineStr">
@@ -27673,116 +27673,6 @@
         </is>
       </c>
       <c r="Q483" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-    </row>
-    <row r="484">
-      <c r="A484" t="inlineStr">
-        <is>
-          <t>Kimi K2 Thinking</t>
-        </is>
-      </c>
-      <c r="B484" t="inlineStr"/>
-      <c r="C484" t="inlineStr"/>
-      <c r="D484" t="inlineStr">
-        <is>
-          <t>月之暗面 (Moonshot AI)</t>
-        </is>
-      </c>
-      <c r="E484" t="inlineStr">
-        <is>
-          <t>国内</t>
-        </is>
-      </c>
-      <c r="F484" t="inlineStr"/>
-      <c r="G484" t="inlineStr"/>
-      <c r="H484" t="inlineStr">
-        <is>
-          <t>推理增强型思考模型</t>
-        </is>
-      </c>
-      <c r="I484" t="inlineStr"/>
-      <c r="J484" t="inlineStr"/>
-      <c r="K484" t="inlineStr"/>
-      <c r="L484" t="inlineStr">
-        <is>
-          <t>虽发布于2025年11月，但在2026年5月30日被量子位等媒体重点报道其‘300轮自主工具调用’能力，并作为K2系列核心组件在2026年5月下旬技术峰会中全面演示，属搜索窗口内关键再曝光模型</t>
-        </is>
-      </c>
-      <c r="M484" t="inlineStr">
-        <is>
-          <t>2025-11-01</t>
-        </is>
-      </c>
-      <c r="N484" t="inlineStr">
-        <is>
-          <t>2026-06-08 03:34</t>
-        </is>
-      </c>
-      <c r="O484" t="inlineStr"/>
-      <c r="P484" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="Q484" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-    </row>
-    <row r="485">
-      <c r="A485" t="inlineStr">
-        <is>
-          <t>Gemini 3.0</t>
-        </is>
-      </c>
-      <c r="B485" t="inlineStr"/>
-      <c r="C485" t="inlineStr"/>
-      <c r="D485" t="inlineStr">
-        <is>
-          <t>Google</t>
-        </is>
-      </c>
-      <c r="E485" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F485" t="inlineStr"/>
-      <c r="G485" t="inlineStr"/>
-      <c r="H485" t="inlineStr">
-        <is>
-          <t>多模态大模型</t>
-        </is>
-      </c>
-      <c r="I485" t="inlineStr"/>
-      <c r="J485" t="inlineStr"/>
-      <c r="K485" t="inlineStr"/>
-      <c r="L485" t="inlineStr">
-        <is>
-          <t>Google正式发布Gemini 3.0，原生支持视频帧级推理、实时语音-文本联合规划，并深度集成Antigravity IDE，为2026年5月底前最新多模态基座模型（权威信源确认其GA发布于5月20日，5月29–31日密集应用披露）</t>
-        </is>
-      </c>
-      <c r="M485" t="inlineStr">
-        <is>
-          <t>2026-05-20</t>
-        </is>
-      </c>
-      <c r="N485" t="inlineStr">
-        <is>
-          <t>2026-06-08 03:34</t>
-        </is>
-      </c>
-      <c r="O485" t="inlineStr"/>
-      <c r="P485" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="Q485" t="inlineStr">
         <is>
           <t>待核实（LLM交叉巡检发现）</t>
         </is>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-06-09
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models.xlsx
+++ b/Model_Navigate/data/Object-Models.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q483"/>
+  <dimension ref="A1:Q486"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27678,6 +27678,183 @@
         </is>
       </c>
     </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>Claude 4.0</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr"/>
+      <c r="C484" t="inlineStr"/>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="E484" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F484" t="inlineStr"/>
+      <c r="G484" t="inlineStr"/>
+      <c r="H484" t="inlineStr">
+        <is>
+          <t>大语言模型</t>
+        </is>
+      </c>
+      <c r="I484" t="inlineStr"/>
+      <c r="J484" t="inlineStr"/>
+      <c r="K484" t="inlineStr">
+        <is>
+          <t>https://www.anthropic.com</t>
+        </is>
+      </c>
+      <c r="L484" t="inlineStr">
+        <is>
+          <t>Anthropic正式发布Claude 4.0，宣称在1M上下文处理、工具调用稳定性及多智能体协同协议（MCP）原生支持方面实现突破，面向企业级Agent工作流深度优化</t>
+        </is>
+      </c>
+      <c r="M484" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="N484" t="inlineStr">
+        <is>
+          <t>2026-06-08 03:34</t>
+        </is>
+      </c>
+      <c r="O484" t="inlineStr">
+        <is>
+          <t>2026-06-09 01:58</t>
+        </is>
+      </c>
+      <c r="P484" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Q484" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>CUA (Contextual Utility Alignment) Training Framework</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr"/>
+      <c r="C485" t="inlineStr"/>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>复旦大学 × 通义实验室</t>
+        </is>
+      </c>
+      <c r="E485" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F485" t="inlineStr"/>
+      <c r="G485" t="inlineStr"/>
+      <c r="H485" t="inlineStr">
+        <is>
+          <t>智能体训练范式 / 方法论</t>
+        </is>
+      </c>
+      <c r="I485" t="inlineStr"/>
+      <c r="J485" t="inlineStr"/>
+      <c r="K485" t="inlineStr"/>
+      <c r="L485" t="inlineStr">
+        <is>
+          <t>提出全新CUA训练范式，解决Agent在复杂Tool选择中的效用对齐问题，非单一模型但已集成至通义千问Qwen-Agent v3.2（同期上线）</t>
+        </is>
+      </c>
+      <c r="M485" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="N485" t="inlineStr">
+        <is>
+          <t>2026-06-08 03:34</t>
+        </is>
+      </c>
+      <c r="O485" t="inlineStr">
+        <is>
+          <t>2026-06-09 01:58</t>
+        </is>
+      </c>
+      <c r="P485" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Q485" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>u2</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr"/>
+      <c r="C486" t="inlineStr"/>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>云知声</t>
+        </is>
+      </c>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F486" t="inlineStr"/>
+      <c r="G486" t="inlineStr"/>
+      <c r="H486" t="inlineStr">
+        <is>
+          <t>原生智能体大语言模型</t>
+        </is>
+      </c>
+      <c r="I486" t="inlineStr"/>
+      <c r="J486" t="inlineStr"/>
+      <c r="K486" t="inlineStr"/>
+      <c r="L486" t="inlineStr">
+        <is>
+          <t>面向个人、开发者与组织的通用大语言模型，具备自主拆解并执行100+步复杂工作流的能力，强调高智能密度与高token价值，在GPQA Diamond（87.9分）和GDPVal（72.5分）等权威评测中进入第一梯队。</t>
+        </is>
+      </c>
+      <c r="M486" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="N486" t="inlineStr">
+        <is>
+          <t>2026-06-09 01:58</t>
+        </is>
+      </c>
+      <c r="O486" t="inlineStr"/>
+      <c r="P486" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Q486" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-06-13
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models.xlsx
+++ b/Model_Navigate/data/Object-Models.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R390"/>
+  <dimension ref="A1:R395"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23135,6 +23135,310 @@
       </c>
       <c r="R390" t="inlineStr"/>
     </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>Kimi K2.7 Code</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr"/>
+      <c r="C391" t="inlineStr"/>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>Moonshot AI</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
+      <c r="G391" t="inlineStr">
+        <is>
+          <t>1T</t>
+        </is>
+      </c>
+      <c r="H391" t="inlineStr">
+        <is>
+          <t>代码</t>
+        </is>
+      </c>
+      <c r="I391" t="inlineStr">
+        <is>
+          <t>thinking</t>
+        </is>
+      </c>
+      <c r="J391" t="inlineStr">
+        <is>
+          <t>通用对话</t>
+        </is>
+      </c>
+      <c r="K391" t="inlineStr">
+        <is>
+          <t>https://llm-stats.com/models/kimi-k2.7-code</t>
+        </is>
+      </c>
+      <c r="L391" t="inlineStr">
+        <is>
+          <t>MoE架构；1T参数；262k上下文；MIT (modified)</t>
+        </is>
+      </c>
+      <c r="M391" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="N391" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="O391" t="inlineStr">
+        <is>
+          <t>2026-06-13 02:09</t>
+        </is>
+      </c>
+      <c r="P391" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="Q391" t="inlineStr">
+        <is>
+          <t>llm-stats.com 排行榜 · HuggingFace 需登录(moonshot-ai/Kimi K2.7 Code)</t>
+        </is>
+      </c>
+      <c r="R391" t="inlineStr"/>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>BAAI Cardiac Agent v1.0</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr"/>
+      <c r="C392" t="inlineStr"/>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>智源研究院</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F392" t="inlineStr"/>
+      <c r="G392" t="inlineStr"/>
+      <c r="H392" t="inlineStr">
+        <is>
+          <t>医疗诊断智能体</t>
+        </is>
+      </c>
+      <c r="I392" t="inlineStr"/>
+      <c r="J392" t="inlineStr"/>
+      <c r="K392" t="inlineStr"/>
+      <c r="L392" t="inlineStr">
+        <is>
+          <t>首个面向心脏磁共振多模态数据的辅助诊断智能体，由智源研究院与安贞医院联合研发，诊断精度达顶尖心血管医生水平。</t>
+        </is>
+      </c>
+      <c r="M392" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="N392" t="inlineStr">
+        <is>
+          <t>2026-06-13 02:10</t>
+        </is>
+      </c>
+      <c r="O392" t="inlineStr"/>
+      <c r="P392" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Q392" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="R392" t="inlineStr"/>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>AREX v1.0</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr"/>
+      <c r="C393" t="inlineStr"/>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>智源研究院</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F393" t="inlineStr"/>
+      <c r="G393" t="inlineStr"/>
+      <c r="H393" t="inlineStr">
+        <is>
+          <t>科学发现智能体</t>
+        </is>
+      </c>
+      <c r="I393" t="inlineStr"/>
+      <c r="J393" t="inlineStr"/>
+      <c r="K393" t="inlineStr"/>
+      <c r="L393" t="inlineStr">
+        <is>
+          <t>面向基础科研全流程的自主研究智能体，支持文献调研、实验设计、结果论证与论文撰写，推动AI驱动的自主科学发现。</t>
+        </is>
+      </c>
+      <c r="M393" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="N393" t="inlineStr">
+        <is>
+          <t>2026-06-13 02:10</t>
+        </is>
+      </c>
+      <c r="O393" t="inlineStr"/>
+      <c r="P393" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Q393" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="R393" t="inlineStr"/>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>SoulAgent v1.0</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr"/>
+      <c r="C394" t="inlineStr"/>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>智源研究院</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr"/>
+      <c r="G394" t="inlineStr"/>
+      <c r="H394" t="inlineStr">
+        <is>
+          <t>个人专属智能体</t>
+        </is>
+      </c>
+      <c r="I394" t="inlineStr"/>
+      <c r="J394" t="inlineStr"/>
+      <c r="K394" t="inlineStr"/>
+      <c r="L394" t="inlineStr">
+        <is>
+          <t>采用自研轻量架构的个人数字分身智能体，Token成本节省30%，资源占用降低80%，支持小程序端即时交互。</t>
+        </is>
+      </c>
+      <c r="M394" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="N394" t="inlineStr">
+        <is>
+          <t>2026-06-13 02:10</t>
+        </is>
+      </c>
+      <c r="O394" t="inlineStr"/>
+      <c r="P394" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Q394" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="R394" t="inlineStr"/>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>RiskGuard Bio-Agent v1.0</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr"/>
+      <c r="C395" t="inlineStr"/>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>智源研究院</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F395" t="inlineStr"/>
+      <c r="G395" t="inlineStr"/>
+      <c r="H395" t="inlineStr">
+        <is>
+          <t>AI安全智能体</t>
+        </is>
+      </c>
+      <c r="I395" t="inlineStr"/>
+      <c r="J395" t="inlineStr"/>
+      <c r="K395" t="inlineStr"/>
+      <c r="L395" t="inlineStr">
+        <is>
+          <t>面向生物安全的风险发现智能体，通过主动模拟攻击者行为，识别有害蛋白序列设计等环节的脆弱性，实现生物风险‘事前演练’防控。</t>
+        </is>
+      </c>
+      <c r="M395" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="N395" t="inlineStr">
+        <is>
+          <t>2026-06-13 02:10</t>
+        </is>
+      </c>
+      <c r="O395" t="inlineStr"/>
+      <c r="P395" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Q395" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="R395" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-06-19
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models.xlsx
+++ b/Model_Navigate/data/Object-Models.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R427"/>
+  <dimension ref="A1:R433"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25355,6 +25355,350 @@
       </c>
       <c r="R427" t="inlineStr"/>
     </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>Lyria 3</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr"/>
+      <c r="C428" t="inlineStr"/>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>Google/DeepMind</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F428" t="inlineStr"/>
+      <c r="G428" t="inlineStr"/>
+      <c r="H428" t="inlineStr">
+        <is>
+          <t>音乐生成模型</t>
+        </is>
+      </c>
+      <c r="I428" t="inlineStr"/>
+      <c r="J428" t="inlineStr"/>
+      <c r="K428" t="inlineStr"/>
+      <c r="L428" t="inlineStr">
+        <is>
+          <t>谷歌发布的第三代端到端音乐生成模型，支持长时序、风格可控、实时交互式创作，集成于Pixel 10a及Wear OS 7</t>
+        </is>
+      </c>
+      <c r="M428" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="N428" t="inlineStr">
+        <is>
+          <t>2026-06-18 02:41</t>
+        </is>
+      </c>
+      <c r="O428" t="inlineStr">
+        <is>
+          <t>2026-06-19 02:50</t>
+        </is>
+      </c>
+      <c r="P428" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Q428" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="R428" t="inlineStr"/>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>京东视觉语言实时交互模型（未命名）</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr"/>
+      <c r="C429" t="inlineStr"/>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>京东</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F429" t="inlineStr"/>
+      <c r="G429" t="inlineStr"/>
+      <c r="H429" t="inlineStr">
+        <is>
+          <t>视觉语言智能体</t>
+        </is>
+      </c>
+      <c r="I429" t="inlineStr"/>
+      <c r="J429" t="inlineStr"/>
+      <c r="K429" t="inlineStr"/>
+      <c r="L429" t="inlineStr">
+        <is>
+          <t>支持摄像头/直播流/监控流+语音I/O的实时流式交互模型，计划开源权重、数据、训练方法及完整系统</t>
+        </is>
+      </c>
+      <c r="M429" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="N429" t="inlineStr">
+        <is>
+          <t>2026-06-18 02:41</t>
+        </is>
+      </c>
+      <c r="O429" t="inlineStr">
+        <is>
+          <t>2026-06-19 02:50</t>
+        </is>
+      </c>
+      <c r="P429" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Q429" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="R429" t="inlineStr"/>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr"/>
+      <c r="C430" t="inlineStr"/>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>MiniMax</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F430" t="inlineStr"/>
+      <c r="G430" t="inlineStr"/>
+      <c r="H430" t="inlineStr">
+        <is>
+          <t>多模态大语言模型</t>
+        </is>
+      </c>
+      <c r="I430" t="inlineStr"/>
+      <c r="J430" t="inlineStr"/>
+      <c r="K430" t="inlineStr"/>
+      <c r="L430" t="inlineStr">
+        <is>
+          <t>MiniMax于6月1日发布的旗舰原生多模态模型，支持150万Token超长上下文、高阶智能体能力，编程评测成绩超越GPT-5.5</t>
+        </is>
+      </c>
+      <c r="M430" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N430" t="inlineStr">
+        <is>
+          <t>2026-06-19 02:51</t>
+        </is>
+      </c>
+      <c r="O430" t="inlineStr"/>
+      <c r="P430" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Q430" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="R430" t="inlineStr"/>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>GPT-5.6</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr"/>
+      <c r="C431" t="inlineStr"/>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F431" t="inlineStr"/>
+      <c r="G431" t="inlineStr"/>
+      <c r="H431" t="inlineStr">
+        <is>
+          <t>大语言模型</t>
+        </is>
+      </c>
+      <c r="I431" t="inlineStr"/>
+      <c r="J431" t="inlineStr"/>
+      <c r="K431" t="inlineStr"/>
+      <c r="L431" t="inlineStr">
+        <is>
+          <t>OpenAI于2026年6月正式发布的GPT-5.6版本，重点优化编码效率与智能体工作流能力，强化企业级权限管控与语音交互支持</t>
+        </is>
+      </c>
+      <c r="M431" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="N431" t="inlineStr">
+        <is>
+          <t>2026-06-19 02:51</t>
+        </is>
+      </c>
+      <c r="O431" t="inlineStr"/>
+      <c r="P431" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Q431" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="R431" t="inlineStr"/>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>Gemini 3.5 Flash</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr"/>
+      <c r="C432" t="inlineStr"/>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>Google/DeepMind</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F432" t="inlineStr"/>
+      <c r="G432" t="inlineStr"/>
+      <c r="H432" t="inlineStr">
+        <is>
+          <t>轻量级多模态大语言模型</t>
+        </is>
+      </c>
+      <c r="I432" t="inlineStr"/>
+      <c r="J432" t="inlineStr"/>
+      <c r="K432" t="inlineStr"/>
+      <c r="L432" t="inlineStr">
+        <is>
+          <t>谷歌I/O 2026推出的极速版模型，专为低延迟智能体服务设计，支撑全天候个人智能体Spark实时响应</t>
+        </is>
+      </c>
+      <c r="M432" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="N432" t="inlineStr">
+        <is>
+          <t>2026-06-19 02:51</t>
+        </is>
+      </c>
+      <c r="O432" t="inlineStr"/>
+      <c r="P432" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Q432" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="R432" t="inlineStr"/>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>Gemma 4 12B</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr"/>
+      <c r="C433" t="inlineStr"/>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>Google/DeepMind</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F433" t="inlineStr"/>
+      <c r="G433" t="inlineStr"/>
+      <c r="H433" t="inlineStr">
+        <is>
+          <t>开源轻量多模态模型</t>
+        </is>
+      </c>
+      <c r="I433" t="inlineStr"/>
+      <c r="J433" t="inlineStr"/>
+      <c r="K433" t="inlineStr"/>
+      <c r="L433" t="inlineStr">
+        <is>
+          <t>谷歌同步开源的12B参数多模态模型，支持原生音频输入，可在普通终端设备本地运行，显著降低AI开发与部署门槛</t>
+        </is>
+      </c>
+      <c r="M433" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="N433" t="inlineStr">
+        <is>
+          <t>2026-06-19 02:51</t>
+        </is>
+      </c>
+      <c r="O433" t="inlineStr"/>
+      <c r="P433" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Q433" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="R433" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-07-01
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models.xlsx
+++ b/Model_Navigate/data/Object-Models.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R467"/>
+  <dimension ref="A1:R469"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27955,6 +27955,158 @@
       </c>
       <c r="R467" t="inlineStr"/>
     </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>Claude Sonnet 5</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr"/>
+      <c r="C468" t="inlineStr"/>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F468" t="inlineStr">
+        <is>
+          <t>闭源</t>
+        </is>
+      </c>
+      <c r="G468" t="inlineStr"/>
+      <c r="H468" t="inlineStr">
+        <is>
+          <t>多模态</t>
+        </is>
+      </c>
+      <c r="I468" t="inlineStr">
+        <is>
+          <t>thinking</t>
+        </is>
+      </c>
+      <c r="J468" t="inlineStr">
+        <is>
+          <t>通用对话</t>
+        </is>
+      </c>
+      <c r="K468" t="inlineStr">
+        <is>
+          <t>https://llm-stats.com/models/claude-sonnet-5</t>
+        </is>
+      </c>
+      <c r="L468" t="inlineStr">
+        <is>
+          <t>1000k上下文；顶级编码能力</t>
+        </is>
+      </c>
+      <c r="M468" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="N468" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="O468" t="inlineStr">
+        <is>
+          <t>2026-07-01 02:13</t>
+        </is>
+      </c>
+      <c r="P468" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="Q468" t="inlineStr">
+        <is>
+          <t>llm-stats.com 排行榜</t>
+        </is>
+      </c>
+      <c r="R468" t="inlineStr"/>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>GELab-Zero-4B-preview-Sico-Evolution</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr"/>
+      <c r="C469" t="inlineStr"/>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>微软</t>
+        </is>
+      </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F469" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
+      <c r="G469" t="inlineStr">
+        <is>
+          <t>4B</t>
+        </is>
+      </c>
+      <c r="H469" t="inlineStr">
+        <is>
+          <t>未知</t>
+        </is>
+      </c>
+      <c r="I469" t="inlineStr">
+        <is>
+          <t>non-thinking</t>
+        </is>
+      </c>
+      <c r="J469" t="inlineStr"/>
+      <c r="K469" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/microsoft/GELab-Zero-4B-preview-Sico-Evolution</t>
+        </is>
+      </c>
+      <c r="L469" t="inlineStr">
+        <is>
+          <t>HuggingFace image-text-to-text</t>
+        </is>
+      </c>
+      <c r="M469" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="N469" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="O469" t="inlineStr">
+        <is>
+          <t>2026-07-01 02:13</t>
+        </is>
+      </c>
+      <c r="P469" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="Q469" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> · HuggingFace 需登录(微软/GELab-Zero-4B-preview-Sico-Evolution)</t>
+        </is>
+      </c>
+      <c r="R469" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>